<commit_message>
starting to implement the gpt network
</commit_message>
<xml_diff>
--- a/documents/time_log.xlsx
+++ b/documents/time_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\user\Uni\BA\BA\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7385AB8-5FA0-4937-82A1-66EDD51147E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0255816F-77C1-463B-B8E1-CAD62E702E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="28800" windowHeight="11295" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
+    <workbookView xWindow="1080" yWindow="1080" windowWidth="28800" windowHeight="11295" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -480,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCFFE4-CAD8-4510-8E64-539F141A23FF}">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
@@ -570,7 +570,7 @@
         <v>7</v>
       </c>
       <c r="Q6">
-        <f t="shared" ref="Q6:Q18" si="0">Q5+B6</f>
+        <f t="shared" ref="Q6:Q19" si="0">Q5+B6</f>
         <v>8.5</v>
       </c>
     </row>
@@ -755,23 +755,38 @@
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>46114</v>
+      </c>
       <c r="B19">
-        <f>SUM(B3:B18)</f>
-        <v>29.75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="0"/>
+        <v>30.75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <f>SUM(B3:B19)</f>
+        <v>30.75</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updating spike gpt implementation
</commit_message>
<xml_diff>
--- a/documents/time_log.xlsx
+++ b/documents/time_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\user\Uni\BA\BA\documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\uni\6. semester\BA Arbeit\BA\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0255816F-77C1-463B-B8E1-CAD62E702E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3370EFEE-F594-4B01-89FE-16490A36F38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="28800" windowHeight="11295" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>implementing the transformer</t>
+  </si>
+  <si>
+    <t>gpt implementation</t>
   </si>
 </sst>
 </file>
@@ -480,13 +483,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCFFE4-CAD8-4510-8E64-539F141A23FF}">
-  <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1"/>
+    <col min="1" max="1" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -500,7 +503,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -514,7 +517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46091</v>
       </c>
@@ -529,7 +532,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>46092</v>
       </c>
@@ -544,7 +547,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>46093</v>
       </c>
@@ -559,7 +562,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>46094</v>
       </c>
@@ -570,11 +573,11 @@
         <v>7</v>
       </c>
       <c r="Q6">
-        <f t="shared" ref="Q6:Q19" si="0">Q5+B6</f>
+        <f t="shared" ref="Q6:Q21" si="0">Q5+B6</f>
         <v>8.5</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>46097</v>
       </c>
@@ -589,7 +592,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>46099</v>
       </c>
@@ -604,7 +607,7 @@
         <v>12.25</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>46100</v>
       </c>
@@ -619,7 +622,7 @@
         <v>13.25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>46101</v>
       </c>
@@ -634,7 +637,7 @@
         <v>14.25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>46102</v>
       </c>
@@ -649,7 +652,7 @@
         <v>15.25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>46103</v>
       </c>
@@ -664,7 +667,7 @@
         <v>19.25</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>46104</v>
       </c>
@@ -679,7 +682,7 @@
         <v>20.75</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>46106</v>
       </c>
@@ -694,7 +697,7 @@
         <v>22.25</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>46108</v>
       </c>
@@ -709,7 +712,7 @@
         <v>22.75</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>46111</v>
       </c>
@@ -724,7 +727,7 @@
         <v>25.75</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>46112</v>
       </c>
@@ -739,7 +742,7 @@
         <v>27.75</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>46113</v>
       </c>
@@ -754,7 +757,7 @@
         <v>29.75</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>46114</v>
       </c>
@@ -769,24 +772,39 @@
         <v>30.75</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>46118</v>
+      </c>
       <c r="B20">
-        <f>SUM(B3:B19)</f>
-        <v>30.75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+        <v>0.5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="0"/>
+        <v>31.25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <f>SUM(B3:B20)</f>
+        <v>31.25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
time update working on compute cluster
</commit_message>
<xml_diff>
--- a/documents/time_log.xlsx
+++ b/documents/time_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\uni\6. semester\BA Arbeit\BA\documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\user\Uni\BA\BA\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3112CD86-3A4C-4583-BDFE-157B6C357F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B5239D-E918-45F4-8AFA-179FFFBF6EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5772" yWindow="0" windowWidth="17280" windowHeight="8964" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
+    <workbookView xWindow="2115" yWindow="2115" windowWidth="28800" windowHeight="11295" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>Date</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>make spike-gpt runable with datacluster dataset. Damn thats hard i can't seem to get it right</t>
+  </si>
+  <si>
+    <t>finally spike-gpt runnable with sbatch</t>
   </si>
 </sst>
 </file>
@@ -486,13 +489,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCFFE4-CAD8-4510-8E64-539F141A23FF}">
-  <dimension ref="A1:Q27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="1"/>
+    <col min="1" max="1" width="11.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,7 +509,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -520,7 +523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46091</v>
       </c>
@@ -535,7 +538,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46092</v>
       </c>
@@ -550,7 +553,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46093</v>
       </c>
@@ -565,7 +568,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46094</v>
       </c>
@@ -576,11 +579,11 @@
         <v>7</v>
       </c>
       <c r="Q6">
-        <f t="shared" ref="Q6:Q21" si="0">Q5+B6</f>
+        <f t="shared" ref="Q6:Q24" si="0">Q5+B6</f>
         <v>8.5</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>46097</v>
       </c>
@@ -595,7 +598,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>46099</v>
       </c>
@@ -610,7 +613,7 @@
         <v>12.25</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>46100</v>
       </c>
@@ -625,7 +628,7 @@
         <v>13.25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>46101</v>
       </c>
@@ -640,7 +643,7 @@
         <v>14.25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>46102</v>
       </c>
@@ -655,7 +658,7 @@
         <v>15.25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>46103</v>
       </c>
@@ -670,7 +673,7 @@
         <v>19.25</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>46104</v>
       </c>
@@ -685,7 +688,7 @@
         <v>20.75</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>46106</v>
       </c>
@@ -700,7 +703,7 @@
         <v>22.25</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>46108</v>
       </c>
@@ -715,7 +718,7 @@
         <v>22.75</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>46111</v>
       </c>
@@ -730,7 +733,7 @@
         <v>25.75</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>46112</v>
       </c>
@@ -745,7 +748,7 @@
         <v>27.75</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>46113</v>
       </c>
@@ -760,7 +763,7 @@
         <v>29.75</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>46114</v>
       </c>
@@ -775,7 +778,7 @@
         <v>30.75</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>46118</v>
       </c>
@@ -790,7 +793,7 @@
         <v>31.25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>46119</v>
       </c>
@@ -805,7 +808,7 @@
         <v>32.75</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>46125</v>
       </c>
@@ -815,25 +818,44 @@
       <c r="C22" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="Q22">
+        <f t="shared" si="0"/>
+        <v>38.75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>46126</v>
+      </c>
       <c r="B23">
-        <f>SUM(B3:B22)</f>
-        <v>38.75</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+        <v>1.5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q23">
+        <f t="shared" si="0"/>
+        <v>40.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <f>SUM(B3:B23)</f>
+        <v>40.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
time log and testFID.py
</commit_message>
<xml_diff>
--- a/documents/time_log.xlsx
+++ b/documents/time_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\uni\6. semester\BA Arbeit\BA\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C02BBA-E140-43C6-814E-598597E65932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B2675E-E0B4-49C0-99C6-30D6BED75A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3396" windowWidth="17280" windowHeight="8964" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A4FDAF27-FB63-47E3-8D62-40C01FCADBEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>Date</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>What is a Brain FID</t>
+  </si>
+  <si>
+    <t>Implement Brain FID</t>
   </si>
 </sst>
 </file>
@@ -510,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCFFE4-CAD8-4510-8E64-539F141A23FF}">
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1"/>
@@ -600,7 +603,7 @@
         <v>7</v>
       </c>
       <c r="Q6">
-        <f t="shared" ref="Q6:Q30" si="0">Q5+B6</f>
+        <f t="shared" ref="Q6:Q31" si="0">Q5+B6</f>
         <v>8.5</v>
       </c>
     </row>
@@ -965,23 +968,38 @@
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>46156</v>
+      </c>
       <c r="B31">
-        <f>SUM(B3:B30)</f>
-        <v>56.75</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q31">
+        <f t="shared" si="0"/>
+        <v>60.75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B37">
+        <f>SUM(B3:B31)</f>
+        <v>60.75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>